<commit_message>
fix table issue from code review; update readme
</commit_message>
<xml_diff>
--- a/tables/results/SuppTable2-Modules.xlsx
+++ b/tables/results/SuppTable2-Modules.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="208">
   <si>
     <t xml:space="preserve"> Module                                                                                                                                                                         </t>
   </si>
@@ -182,7 +182,10 @@
     <t xml:space="preserve"> `histologies.tsv`   `fusion-putative-oncogenic.tsv`   `fusion-dgd.tsv.gz`   `independent-specimens.rnaseqpanel.primary.tsv`  `independent-specimens.rnaseqpanel.relapse.tsv`   `independent-specimens.rnaseqpanel.primary.eachcohort.tsv`   `independent-specimens.rnaseqpanel.relapse.eachcohort.tsv`                                                                                                                                                                                                                                                                                                                                                                                                                                                                           </t>
   </si>
   <si>
-    <t xml:space="preserve"> Gathers counts and frequencies for fusion per cancer_group and cohort                                                                                                                                                                                                                  </t>
+    <t xml:space="preserve"> Gathers counts and frequencies for fusion per cancer_group and cohort                  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> No                                                                                                                                                                                                </t>
   </si>
   <si>
     <t xml:space="preserve"> `results/putative-oncogene-fused-gene-freq.jsonl.gz`   `results/putative-oncogene-fused-gene-freq.tsv.gz`   `results/putative-oncogene-fusion-freq.jsonl.gz`   `results/putative-oncogene-fusion-freq.tsv.gz` </t>
@@ -1196,103 +1199,103 @@
         <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>13</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
         <v>24</v>
       </c>
       <c r="E15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
         <v>24</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D17" t="s">
         <v>8</v>
       </c>
       <c r="E17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
         <v>8</v>
       </c>
       <c r="E18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
         <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D20" t="s">
         <v>8</v>
@@ -1303,30 +1306,30 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D21" t="s">
         <v>8</v>
       </c>
       <c r="E21" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D22" t="s">
         <v>8</v>
@@ -1337,13 +1340,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B23" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D23" t="s">
         <v>8</v>
@@ -1354,132 +1357,132 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B24" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C24" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D24" t="s">
         <v>8</v>
       </c>
       <c r="E24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B25" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C25" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D25" t="s">
         <v>8</v>
       </c>
       <c r="E25" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
         <v>8</v>
       </c>
       <c r="E26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D27" t="s">
         <v>8</v>
       </c>
       <c r="E27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B28" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C28" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D28" t="s">
         <v>8</v>
       </c>
       <c r="E28" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D29" t="s">
         <v>8</v>
       </c>
       <c r="E29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D30" t="s">
         <v>8</v>
       </c>
       <c r="E30" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C31" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D31" t="s">
         <v>8</v>
@@ -1490,115 +1493,115 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B32" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D32" t="s">
         <v>8</v>
       </c>
       <c r="E32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D33" t="s">
         <v>8</v>
       </c>
       <c r="E33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D34" t="s">
         <v>8</v>
       </c>
       <c r="E34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B35" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D35" t="s">
         <v>8</v>
       </c>
       <c r="E35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B36" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C36" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D36" t="s">
         <v>8</v>
       </c>
       <c r="E36" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C37" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D37" t="s">
         <v>8</v>
       </c>
       <c r="E37" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B38" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C38" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D38" t="s">
         <v>8</v>
@@ -1609,13 +1612,13 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B39" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C39" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D39" t="s">
         <v>8</v>
@@ -1626,13 +1629,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D40" t="s">
         <v>8</v>
@@ -1643,13 +1646,13 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B41" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C41" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D41" t="s">
         <v>8</v>
@@ -1660,64 +1663,64 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B42" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C42" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D42" t="s">
         <v>24</v>
       </c>
       <c r="E42" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B43" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C43" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D43" t="s">
         <v>24</v>
       </c>
       <c r="E43" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B44" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C44" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D44" t="s">
         <v>8</v>
       </c>
       <c r="E44" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B45" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C45" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D45" t="s">
         <v>24</v>
@@ -1728,64 +1731,64 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B46" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C46" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D46" t="s">
         <v>8</v>
       </c>
       <c r="E46" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B47" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D47" t="s">
         <v>24</v>
       </c>
       <c r="E47" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B48" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C48" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D48" t="s">
         <v>8</v>
       </c>
       <c r="E48" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B49" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C49" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D49" t="s">
         <v>8</v>
@@ -1796,64 +1799,64 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B50" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C50" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D50" t="s">
         <v>8</v>
       </c>
       <c r="E50" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B51" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C51" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D51" t="s">
         <v>24</v>
       </c>
       <c r="E51" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B52" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C52" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D52" t="s">
         <v>8</v>
       </c>
       <c r="E52" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B53" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C53" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D53" t="s">
         <v>8</v>
@@ -1864,30 +1867,30 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B54" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C54" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D54" t="s">
         <v>8</v>
       </c>
       <c r="E54" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B55" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C55" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D55" t="s">
         <v>8</v>

</xml_diff>